<commit_message>
Campaign draft: copy, rewards, fulfillment plan, video script, graphics, research
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TmekonzsErK6cW9QseAGS5
</commit_message>
<xml_diff>
--- a/kickstarter-campaign/03_financial_model/WW_Kickstarter_Financial_Model_v1.xlsx
+++ b/kickstarter-campaign/03_financial_model/WW_Kickstarter_Financial_Model_v1.xlsx
@@ -989,7 +989,7 @@
         </is>
       </c>
       <c r="B18" s="10" t="n">
-        <v>4950</v>
+        <v>4699</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
@@ -998,14 +998,14 @@
       </c>
       <c r="D18" s="6" t="inlineStr">
         <is>
-          <t>10% below $5,500 target MSRP; rewards first movers without undercutting Northern Tool MAP long term</t>
+          <t>6% below the $4,999 MAP proposed on the Northern Tool quote sheet (2026-09-12 packet); rewards first movers; limited to 10</t>
         </is>
       </c>
       <c r="E18" s="11" t="n">
-        <v>4750</v>
+        <v>4499</v>
       </c>
       <c r="F18" s="11" t="n">
-        <v>5100</v>
+        <v>4999</v>
       </c>
     </row>
     <row r="19">
@@ -1015,7 +1015,7 @@
         </is>
       </c>
       <c r="B19" s="10" t="n">
-        <v>5250</v>
+        <v>4999</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
@@ -1024,14 +1024,14 @@
       </c>
       <c r="D19" s="6" t="inlineStr">
         <is>
-          <t>~4.5% below target MSRP $5,500</t>
+          <t>Equal to the $4,999 MAP proposed to Northern Tool, so the campaign never undercuts a future retail partner</t>
         </is>
       </c>
       <c r="E19" s="11" t="n">
-        <v>5100</v>
+        <v>4799</v>
       </c>
       <c r="F19" s="11" t="n">
-        <v>5500</v>
+        <v>5499</v>
       </c>
     </row>
     <row r="20">
@@ -1041,7 +1041,7 @@
         </is>
       </c>
       <c r="B20" s="10" t="n">
-        <v>5900</v>
+        <v>5599</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
@@ -1050,14 +1050,14 @@
       </c>
       <c r="D20" s="6" t="inlineStr">
         <is>
-          <t>Pump + 2 in. discharge hose (50 ft), adjustable nozzle, suction hose, strainer, spare fob</t>
+          <t>Kickstarter price + $600 package: 2 in. discharge hose (50 ft), adjustable nozzle, suction hose, strainer, spare fob</t>
         </is>
       </c>
       <c r="E20" s="11" t="n">
-        <v>5750</v>
+        <v>5399</v>
       </c>
       <c r="F20" s="11" t="n">
-        <v>6100</v>
+        <v>5899</v>
       </c>
     </row>
     <row r="21">
@@ -1076,7 +1076,7 @@
       </c>
       <c r="D21" s="6" t="inlineStr">
         <is>
-          <t>Palletized ~180 lb crate; LTL residential+liftgate quotes typically $250–$450 from Bend OR</t>
+          <t>Packed 40×28×24 in, 165 lb per Northern Tool quote sheet (2026-09-12); LTL residential + liftgate from Bend OR typically $250–$450; get 2 carrier quotes</t>
         </is>
       </c>
       <c r="E21" s="11" t="n">
@@ -1622,16 +1622,16 @@
         </is>
       </c>
       <c r="B48" s="10" t="n">
-        <v>4598</v>
+        <v>10598</v>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>VERIFIED</t>
+          <t>VERIFIED (quote)</t>
         </is>
       </c>
       <c r="D48" s="6" t="inlineStr">
         <is>
-          <t>Kinsale GL quote 2026-09-01 #07520376: $4,597.91 paid in full ($1M/$2M). Not yet bound. Alternative StarStone quote $10,598 ($2M/$4M)</t>
+          <t>StarStone via RPS: $10,598.05, $2M/$4M occurrence (the limits Northern Tool requires; business plan 2026-09-15 budgets this). Alternative Kinsale quote 2026-09-01 #07520376: $4,597.91 ($1M/$2M claims-made). Neither bound.</t>
         </is>
       </c>
       <c r="E48" s="11" t="n">
@@ -4247,11 +4247,11 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>StarStone insurance ($10,598) instead of Kinsale</t>
+          <t>Kinsale insurance ($4,598) instead of StarStone</t>
         </is>
       </c>
       <c r="B7" s="11">
-        <f>Scenarios!C31-(10598-o_insur)</f>
+        <f>Scenarios!C31+(o_insur-4598)</f>
         <v/>
       </c>
       <c r="C7" s="11">
@@ -4260,7 +4260,7 @@
       </c>
       <c r="D7" s="6" t="inlineStr">
         <is>
-          <t>If $2M/$4M limits are required by a retailer</t>
+          <t>If $1M/$2M claims-made is accepted for a direct-sales-only year</t>
         </is>
       </c>
     </row>

</xml_diff>